<commit_message>
Updated with bug report
</commit_message>
<xml_diff>
--- a/saucedemo-manual-testing/Test-Cases/test-cases.xlsx
+++ b/saucedemo-manual-testing/Test-Cases/test-cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fazz Com 03364446969\Desktop\qa-testing-project\Test-Cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fazz Com 03364446969\Desktop\qa-testing-project\saucedemo-manual-testing\Test-Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3604BCB4-49D8-491A-A7D4-B80A037DFC3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70FE2648-42B0-4C9A-BA16-D1F43490BB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5C3CFA41-E3BE-4C4B-8BE1-10660847915D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="153">
   <si>
     <t>Website Name</t>
   </si>
@@ -481,6 +481,9 @@
   </si>
   <si>
     <t>Failed</t>
+  </si>
+  <si>
+    <t>https://snipboard.io/itbjP0.jpg</t>
   </si>
 </sst>
 </file>
@@ -629,7 +632,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -656,10 +659,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -680,6 +679,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1021,7 +1021,7 @@
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>142</v>
       </c>
     </row>
@@ -1032,8 +1032,11 @@
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="10" t="s">
         <v>143</v>
+      </c>
+      <c r="H2" s="17">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="19.8" x14ac:dyDescent="0.55000000000000004">
@@ -1043,8 +1046,11 @@
       <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G3" s="12" t="s">
         <v>144</v>
+      </c>
+      <c r="H3" s="17">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="19.8" x14ac:dyDescent="0.55000000000000004">
@@ -1054,10 +1060,10 @@
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="17">
         <v>29</v>
       </c>
     </row>
@@ -1134,7 +1140,7 @@
         <v>146</v>
       </c>
       <c r="H10" s="8"/>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="14" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1161,7 +1167,7 @@
         <v>146</v>
       </c>
       <c r="H11" s="8"/>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="14" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1187,11 +1193,11 @@
       <c r="G12" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="I12" s="18" t="s">
-        <v>151</v>
+      <c r="I12" s="14" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1213,9 +1219,13 @@
       <c r="F13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="8"/>
+      <c r="G13" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="I13" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -1236,9 +1246,13 @@
       <c r="F14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="I14" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
@@ -1259,9 +1273,13 @@
       <c r="F15" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="8"/>
+      <c r="G15" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+      <c r="I15" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
@@ -1293,9 +1311,13 @@
       <c r="F17" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G17" s="8"/>
+      <c r="G17" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
+      <c r="I17" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
@@ -1316,9 +1338,13 @@
       <c r="F18" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="G18" s="8"/>
+      <c r="G18" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
+      <c r="I18" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
@@ -1339,9 +1365,13 @@
       <c r="F19" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="8"/>
+      <c r="G19" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="I19" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
@@ -1362,9 +1392,13 @@
       <c r="F20" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="G20" s="8"/>
+      <c r="G20" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+      <c r="I20" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
@@ -1385,9 +1419,13 @@
       <c r="F21" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="8"/>
+      <c r="G21" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="I21" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
@@ -1408,9 +1446,13 @@
       <c r="F22" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="G22" s="8"/>
+      <c r="G22" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="I22" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
@@ -1442,9 +1484,13 @@
       <c r="F24" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="G24" s="8"/>
+      <c r="G24" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="I24" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
@@ -1465,9 +1511,13 @@
       <c r="F25" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="8"/>
+      <c r="G25" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="I25" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
@@ -1488,9 +1538,13 @@
       <c r="F26" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="G26" s="8"/>
+      <c r="G26" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
+      <c r="I26" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
@@ -1511,9 +1565,13 @@
       <c r="F27" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="G27" s="8"/>
+      <c r="G27" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
+      <c r="I27" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
@@ -1545,9 +1603,13 @@
       <c r="F29" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="8"/>
+      <c r="G29" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
+      <c r="I29" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
@@ -1568,9 +1630,15 @@
       <c r="F30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
+      <c r="G30" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H30" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="I30" s="16" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
@@ -1591,9 +1659,13 @@
       <c r="F31" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G31" s="8"/>
+      <c r="G31" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
+      <c r="I31" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
@@ -1614,9 +1686,13 @@
       <c r="F32" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="G32" s="8"/>
+      <c r="G32" s="8" t="s">
+        <v>149</v>
+      </c>
       <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
+      <c r="I32" s="16" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
@@ -1637,9 +1713,13 @@
       <c r="F33" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="G33" s="8"/>
+      <c r="G33" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
+      <c r="I33" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
@@ -1660,9 +1740,13 @@
       <c r="F34" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="G34" s="8"/>
+      <c r="G34" s="8" t="s">
+        <v>149</v>
+      </c>
       <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
+      <c r="I34" s="16" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
@@ -1683,9 +1767,13 @@
       <c r="F35" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="G35" s="8"/>
+      <c r="G35" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
+      <c r="I35" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
@@ -1717,9 +1805,13 @@
       <c r="F37" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="G37" s="8"/>
+      <c r="G37" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
+      <c r="I37" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
@@ -1740,9 +1832,13 @@
       <c r="F38" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="G38" s="8"/>
+      <c r="G38" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
+      <c r="I38" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
@@ -1763,9 +1859,13 @@
       <c r="F39" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="G39" s="8"/>
+      <c r="G39" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
+      <c r="I39" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
@@ -1797,9 +1897,13 @@
       <c r="F41" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="G41" s="8"/>
+      <c r="G41" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
+      <c r="I41" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
@@ -1820,39 +1924,48 @@
       <c r="F42" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="G42" s="8"/>
+      <c r="G42" s="8" t="s">
+        <v>146</v>
+      </c>
       <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
+      <c r="I42" s="14" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="10" t="s">
+      <c r="A43" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="F43" s="11" t="s">
+      <c r="F43" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="G43" s="8"/>
+      <c r="G43" s="8" t="s">
+        <v>149</v>
+      </c>
       <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
+      <c r="I43" s="16" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B1" r:id="rId1" xr:uid="{C1475E8B-DF2B-4F19-A42B-9E740EBF05E3}"/>
     <hyperlink ref="H12" r:id="rId2" xr:uid="{2E12DB04-A88B-40FA-BC48-F640A79A4DDE}"/>
+    <hyperlink ref="H30" r:id="rId3" xr:uid="{BF0477FE-19E6-4EE2-B7AB-43DCFAD60316}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>